<commit_message>
Updated parameters with better assumptions
</commit_message>
<xml_diff>
--- a/CarData.xlsx
+++ b/CarData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pmull\Documents\MATLAB\Suspension-MATLAB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3166B261-DF63-4865-B65A-6F99A5CD2A26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBEB7ABB-C153-483D-9D84-5B9449E686C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8E514F0D-2B4B-4F97-9824-AFB3030C5F31}"/>
+    <workbookView xWindow="5475" yWindow="2505" windowWidth="21600" windowHeight="11835" xr2:uid="{8E514F0D-2B4B-4F97-9824-AFB3030C5F31}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>Spring Rate</t>
   </si>
@@ -83,9 +83,6 @@
     <t>Sprung weight</t>
   </si>
   <si>
-    <t>assuming 30lbs per corner</t>
-  </si>
-  <si>
     <t>MR</t>
   </si>
   <si>
@@ -95,9 +92,6 @@
     <t>Roll Center Height</t>
   </si>
   <si>
-    <t>subject to change</t>
-  </si>
-  <si>
     <t>Wheelbase</t>
   </si>
   <si>
@@ -113,13 +107,13 @@
     <t>lb/in assumed</t>
   </si>
   <si>
-    <t>assuming</t>
-  </si>
-  <si>
     <t>Tire Radius</t>
   </si>
   <si>
     <t>in radius</t>
+  </si>
+  <si>
+    <t>&lt;- NOT NEEDED</t>
   </si>
 </sst>
 </file>
@@ -161,15 +155,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -553,7 +546,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.140625" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="5" max="5" width="14.85546875" customWidth="1"/>
     <col min="6" max="6" width="23.140625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -577,26 +570,23 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B2" s="3"/>
-    </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3">
         <f>D3*E3</f>
-        <v>261</v>
+        <v>232</v>
       </c>
       <c r="C3">
         <f>D3-B3</f>
-        <v>319</v>
-      </c>
-      <c r="D3" s="5">
+        <v>348</v>
+      </c>
+      <c r="D3" s="4">
         <v>580</v>
       </c>
       <c r="E3" s="1">
-        <v>0.45</v>
+        <v>0.4</v>
       </c>
       <c r="F3" t="s">
         <v>4</v>
@@ -606,27 +596,22 @@
       <c r="A4" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="3"/>
       <c r="D4" s="2">
-        <v>30</v>
-      </c>
-      <c r="F4" t="s">
-        <v>13</v>
+        <v>448</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="3"/>
       <c r="D5" s="2"/>
-      <c r="E5" s="4"/>
+      <c r="E5" s="3"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" s="3">
+        <v>17</v>
+      </c>
+      <c r="B6">
         <f>D10*((B7)^2)</f>
         <v>150</v>
       </c>
@@ -635,39 +620,38 @@
         <v>150</v>
       </c>
       <c r="F6" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="7">
+        <v>13</v>
+      </c>
+      <c r="B7" s="4">
         <v>1</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="4">
         <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" s="3"/>
-      <c r="D8">
+        <v>16</v>
+      </c>
+      <c r="D8" s="5">
         <f>[1]Front!$B$18</f>
         <v>63.5</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9">
+        <v>14</v>
+      </c>
+      <c r="B9" s="5">
         <f>[1]Front!$B$9</f>
         <v>45.43</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="5">
         <f>[1]Rear!$B$8</f>
         <v>43.43</v>
       </c>
@@ -687,18 +671,15 @@
       <c r="A11" t="s">
         <v>5</v>
       </c>
-      <c r="D11" s="5">
-        <v>10</v>
-      </c>
-      <c r="F11" t="s">
-        <v>23</v>
+      <c r="D11" s="4">
+        <v>13</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12">
+        <v>15</v>
+      </c>
+      <c r="B12" s="5">
         <f>[1]Front!$B$10</f>
         <v>2.6</v>
       </c>
@@ -706,30 +687,30 @@
         <f>_xlfn.REGEXREPLACE([1]Rear!$B$9, "[^0-9.]", "") +0</f>
         <v>5.0999999999999996</v>
       </c>
-      <c r="F12" t="s">
-        <v>17</v>
-      </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>21</v>
-      </c>
-      <c r="D14" s="5">
+        <v>19</v>
+      </c>
+      <c r="D14" s="4">
         <v>480</v>
       </c>
+      <c r="E14" t="s">
+        <v>23</v>
+      </c>
       <c r="F14" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>24</v>
-      </c>
-      <c r="D15">
-        <v>10</v>
+        <v>21</v>
+      </c>
+      <c r="D15" s="4">
+        <v>8</v>
       </c>
       <c r="F15" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>